<commit_message>
4주차 PIT -2.5 0.5u 체결가 정정: Polymarket 52c(≈-108)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/NFL_픽_추적기.xlsx
+++ b/data/NFL_픽_추적기.xlsx
@@ -3230,7 +3230,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>-120</t>
+          <t>-108</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -3256,7 +3256,7 @@
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>Paul 자체 판단 0.5u — 발행 판단은 패스(굳이 하나만 PIT -2.5). 배당 미확인 — 발행 시점 시장가 -120 으로 임시(Paul 확인 시 정정). Ramsey(PIT CB) Q 상태에서 베팅</t>
+          <t>Paul 자체 판단 0.5u — 발행 판단은 패스(굳이 하나만 PIT -2.5). 체결 Polymarket 「PIT to win by over 2.5 → Yes」 52c(≈ -108, 손익분기 52.0%). Ramsey(PIT CB) Q 상태에서 베팅</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">

</xml_diff>

<commit_message>
4주차 목요일 리프레시 10/1 15:52판 + PIT@CLE 채점(CLE 27-24 — 실베팅 PIT -2.5 0.5u L · 방향 PIT -2.5 L/Over W · 티저 다리 CLE +8.5 W)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/NFL_픽_추적기.xlsx
+++ b/data/NFL_픽_추적기.xlsx
@@ -2536,11 +2536,11 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Over 47.5</t>
+          <t>Over 48.5</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>47.5</v>
+        <v>48.5</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -2561,10 +2561,10 @@
         <v>56</v>
       </c>
       <c r="J33" t="n">
-        <v>8.5</v>
+        <v>7.5</v>
       </c>
       <c r="K33" t="n">
-        <v>79</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
@@ -2878,11 +2878,11 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>NE +6.5</t>
+          <t>NE +7</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>-6.5</v>
+        <v>-7</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -2903,10 +2903,10 @@
         <v>2.9</v>
       </c>
       <c r="J39" t="n">
-        <v>-3.6</v>
+        <v>-4.1</v>
       </c>
       <c r="K39" t="n">
-        <v>60.8</v>
+        <v>62.3</v>
       </c>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
@@ -3130,9 +3130,19 @@
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr"/>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>PIT 24-27 CLE</t>
+        </is>
+      </c>
+      <c r="N43" t="n">
+        <v>0.37</v>
+      </c>
       <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr">
         <is>
@@ -3191,9 +3201,19 @@
       <c r="K44" t="n">
         <v>56.9</v>
       </c>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>PIT 24-27 CLE</t>
+        </is>
+      </c>
+      <c r="N44" t="n">
+        <v>-1</v>
+      </c>
       <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr">
         <is>
@@ -3246,9 +3266,19 @@
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>PIT 24-27 CLE</t>
+        </is>
+      </c>
+      <c r="N45" t="n">
+        <v>-0.5</v>
+      </c>
       <c r="O45" t="inlineStr">
         <is>
           <t>2026-10-01 11:36</t>
@@ -3311,9 +3341,19 @@
       <c r="K46" t="n">
         <v>65.8</v>
       </c>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>PIT 24-27 CLE</t>
+        </is>
+      </c>
+      <c r="N46" t="n">
+        <v>-1</v>
+      </c>
       <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr"/>
       <c r="Q46" t="inlineStr">
@@ -3368,9 +3408,19 @@
       <c r="K47" t="n">
         <v>65.8</v>
       </c>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>PIT 24-27 CLE</t>
+        </is>
+      </c>
+      <c r="N47" t="n">
+        <v>0.909</v>
+      </c>
       <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr">
         <is>
@@ -3564,13 +3614,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -3579,7 +3629,7 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>-2</v>
+        <v>-2.5</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -3621,19 +3671,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
+      <c r="F4" t="n">
+        <v>50</v>
+      </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>-0.09</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -3648,22 +3701,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C5" t="n">
         <v>11</v>
       </c>
       <c r="D5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>57.9</v>
+        <v>55</v>
       </c>
       <c r="G5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -3678,10 +3731,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -3689,12 +3742,15 @@
       <c r="E6" t="n">
         <v>0</v>
       </c>
+      <c r="F6" t="n">
+        <v>100</v>
+      </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>0.37</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>웡 티저 다리(10/1~) — 손익분기 73.9%(−120 2팀 환산) · 60다리 보고 · &lt;72% 폐기</t>
+          <t>웡 티저 다리(10/1~) — 손익분기 73.9%(−120 2팀 환산) · 60다리 보고 · &lt;72% 폐기 · 평균 표시가 73.0c(n 1)</t>
         </is>
       </c>
     </row>
@@ -3732,7 +3788,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C8" t="n">
         <v>1</v>
@@ -3741,10 +3797,10 @@
         <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G8" t="n">
-        <v>0.5</v>
+        <v>0.33</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -3783,7 +3839,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
@@ -3792,6 +3848,9 @@
         <v>0</v>
       </c>
       <c r="E10" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" t="n">
         <v>0</v>
       </c>
       <c r="H10" t="inlineStr">
@@ -3838,13 +3897,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C14" t="n">
         <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
@@ -3853,7 +3912,7 @@
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>-1</v>
+        <v>-1.5</v>
       </c>
       <c r="H14" t="inlineStr"/>
     </row>
@@ -3923,13 +3982,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C18" t="n">
         <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
@@ -3938,7 +3997,7 @@
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>-1</v>
+        <v>-1.5</v>
       </c>
       <c r="H18" t="inlineStr"/>
     </row>
@@ -3956,22 +4015,22 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="G21" t="n">
-        <v>-2</v>
+        <v>-2.13</v>
       </c>
       <c r="H21" t="inlineStr"/>
     </row>
@@ -3982,22 +4041,22 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C22" t="n">
         <v>1</v>
       </c>
       <c r="D22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>33.3</v>
+        <v>25</v>
       </c>
       <c r="G22" t="n">
-        <v>-1.09</v>
+        <v>-2.09</v>
       </c>
       <c r="H22" t="inlineStr"/>
     </row>
@@ -4008,22 +4067,22 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C23" t="n">
+        <v>5</v>
+      </c>
+      <c r="D23" t="n">
         <v>4</v>
       </c>
-      <c r="D23" t="n">
-        <v>3</v>
-      </c>
       <c r="E23" t="n">
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>57.1</v>
+        <v>55.6</v>
       </c>
       <c r="G23" t="n">
-        <v>0.64</v>
+        <v>0.55</v>
       </c>
       <c r="H23" t="inlineStr"/>
     </row>
@@ -4064,7 +4123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4172,6 +4231,44 @@
         <v>0</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
4주차 채점 마감 10/06(MNF ATL@NO 포함 16경기)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/NFL_픽_추적기.xlsx
+++ b/data/NFL_픽_추적기.xlsx
@@ -3357,9 +3357,19 @@
       <c r="K44" t="n">
         <v>67.7</v>
       </c>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>ARI 24-36 NYG</t>
+        </is>
+      </c>
+      <c r="N44" t="n">
+        <v>0.909</v>
+      </c>
       <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr"/>
       <c r="Q44" t="inlineStr">
@@ -3550,9 +3560,19 @@
       <c r="K47" t="n">
         <v>72.40000000000001</v>
       </c>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>ARI 24-36 NYG</t>
+        </is>
+      </c>
+      <c r="N47" t="n">
+        <v>0.909</v>
+      </c>
       <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr"/>
       <c r="Q47" t="inlineStr">
@@ -3672,9 +3692,19 @@
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>ATL 45-24 NO</t>
+        </is>
+      </c>
+      <c r="N49" t="n">
+        <v>0.353</v>
+      </c>
       <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr">
         <is>
@@ -3727,9 +3757,19 @@
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr"/>
       <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>ATL 45-24 NO</t>
+        </is>
+      </c>
+      <c r="N50" t="n">
+        <v>-1</v>
+      </c>
       <c r="O50" t="inlineStr"/>
       <c r="P50" t="inlineStr">
         <is>
@@ -3788,9 +3828,19 @@
       <c r="K51" t="n">
         <v>79.3</v>
       </c>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>ATL 45-24 NO</t>
+        </is>
+      </c>
+      <c r="N51" t="n">
+        <v>-1</v>
+      </c>
       <c r="O51" t="inlineStr"/>
       <c r="P51" t="inlineStr"/>
       <c r="Q51" t="inlineStr">
@@ -3845,9 +3895,19 @@
       <c r="K52" t="n">
         <v>79.3</v>
       </c>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>ATL 45-24 NO</t>
+        </is>
+      </c>
+      <c r="N52" t="n">
+        <v>0.909</v>
+      </c>
       <c r="O52" t="inlineStr"/>
       <c r="P52" t="inlineStr">
         <is>
@@ -3973,9 +4033,19 @@
       <c r="K54" t="n">
         <v>62.4</v>
       </c>
-      <c r="L54" t="inlineStr"/>
-      <c r="M54" t="inlineStr"/>
-      <c r="N54" t="inlineStr"/>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>DAL 34-30 HOU</t>
+        </is>
+      </c>
+      <c r="N54" t="n">
+        <v>-1</v>
+      </c>
       <c r="O54" t="inlineStr"/>
       <c r="P54" t="inlineStr"/>
       <c r="Q54" t="inlineStr">
@@ -4166,9 +4236,19 @@
       <c r="K57" t="n">
         <v>75.7</v>
       </c>
-      <c r="L57" t="inlineStr"/>
-      <c r="M57" t="inlineStr"/>
-      <c r="N57" t="inlineStr"/>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>DAL 34-30 HOU</t>
+        </is>
+      </c>
+      <c r="N57" t="n">
+        <v>0.909</v>
+      </c>
       <c r="O57" t="inlineStr"/>
       <c r="P57" t="inlineStr"/>
       <c r="Q57" t="inlineStr">
@@ -4359,9 +4439,19 @@
       <c r="K60" t="n">
         <v>75.2</v>
       </c>
-      <c r="L60" t="inlineStr"/>
-      <c r="M60" t="inlineStr"/>
-      <c r="N60" t="inlineStr"/>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>DEN 14-24 SF</t>
+        </is>
+      </c>
+      <c r="N60" t="n">
+        <v>-1</v>
+      </c>
       <c r="O60" t="inlineStr"/>
       <c r="P60" t="inlineStr"/>
       <c r="Q60" t="inlineStr">
@@ -4552,9 +4642,19 @@
       <c r="K63" t="n">
         <v>56.7</v>
       </c>
-      <c r="L63" t="inlineStr"/>
-      <c r="M63" t="inlineStr"/>
-      <c r="N63" t="inlineStr"/>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>DET 26-32 CAR</t>
+        </is>
+      </c>
+      <c r="N63" t="n">
+        <v>0.909</v>
+      </c>
       <c r="O63" t="inlineStr"/>
       <c r="P63" t="inlineStr"/>
       <c r="Q63" t="inlineStr">
@@ -4674,9 +4774,19 @@
       <c r="K65" t="n">
         <v>68.2</v>
       </c>
-      <c r="L65" t="inlineStr"/>
-      <c r="M65" t="inlineStr"/>
-      <c r="N65" t="inlineStr"/>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>DET 26-32 CAR</t>
+        </is>
+      </c>
+      <c r="N65" t="n">
+        <v>0.909</v>
+      </c>
       <c r="O65" t="inlineStr"/>
       <c r="P65" t="inlineStr"/>
       <c r="Q65" t="inlineStr">
@@ -4731,9 +4841,19 @@
       <c r="K66" t="n">
         <v>58.6</v>
       </c>
-      <c r="L66" t="inlineStr"/>
-      <c r="M66" t="inlineStr"/>
-      <c r="N66" t="inlineStr"/>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>GB 17-14 TB</t>
+        </is>
+      </c>
+      <c r="N66" t="n">
+        <v>0</v>
+      </c>
       <c r="O66" t="inlineStr"/>
       <c r="P66" t="inlineStr"/>
       <c r="Q66" t="inlineStr">
@@ -4859,9 +4979,19 @@
       <c r="K68" t="n">
         <v>65.09999999999999</v>
       </c>
-      <c r="L68" t="inlineStr"/>
-      <c r="M68" t="inlineStr"/>
-      <c r="N68" t="inlineStr"/>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>GB 17-14 TB</t>
+        </is>
+      </c>
+      <c r="N68" t="n">
+        <v>-1</v>
+      </c>
       <c r="O68" t="inlineStr"/>
       <c r="P68" t="inlineStr"/>
       <c r="Q68" t="inlineStr">
@@ -4987,9 +5117,19 @@
       <c r="K70" t="n">
         <v>68.2</v>
       </c>
-      <c r="L70" t="inlineStr"/>
-      <c r="M70" t="inlineStr"/>
-      <c r="N70" t="inlineStr"/>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>IND 30-13 WAS</t>
+        </is>
+      </c>
+      <c r="N70" t="n">
+        <v>0.909</v>
+      </c>
       <c r="O70" t="inlineStr"/>
       <c r="P70" t="inlineStr"/>
       <c r="Q70" t="inlineStr">
@@ -5178,9 +5318,19 @@
       <c r="K73" t="n">
         <v>82.8</v>
       </c>
-      <c r="L73" t="inlineStr"/>
-      <c r="M73" t="inlineStr"/>
-      <c r="N73" t="inlineStr"/>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>JAX 22-17 CIN</t>
+        </is>
+      </c>
+      <c r="N73" t="n">
+        <v>0.909</v>
+      </c>
       <c r="O73" t="inlineStr"/>
       <c r="P73" t="inlineStr"/>
       <c r="Q73" t="inlineStr">
@@ -5509,9 +5659,19 @@
       <c r="K78" t="n">
         <v>65.09999999999999</v>
       </c>
-      <c r="L78" t="inlineStr"/>
-      <c r="M78" t="inlineStr"/>
-      <c r="N78" t="inlineStr"/>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>KC 30-27 LV</t>
+        </is>
+      </c>
+      <c r="N78" t="n">
+        <v>-1</v>
+      </c>
       <c r="O78" t="inlineStr"/>
       <c r="P78" t="inlineStr"/>
       <c r="Q78" t="inlineStr">
@@ -5637,9 +5797,19 @@
       <c r="K80" t="n">
         <v>72.5</v>
       </c>
-      <c r="L80" t="inlineStr"/>
-      <c r="M80" t="inlineStr"/>
-      <c r="N80" t="inlineStr"/>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>KC 30-27 LV</t>
+        </is>
+      </c>
+      <c r="N80" t="n">
+        <v>-1</v>
+      </c>
       <c r="O80" t="inlineStr"/>
       <c r="P80" t="inlineStr"/>
       <c r="Q80" t="inlineStr">
@@ -5830,9 +6000,19 @@
       <c r="K83" t="n">
         <v>62.1</v>
       </c>
-      <c r="L83" t="inlineStr"/>
-      <c r="M83" t="inlineStr"/>
-      <c r="N83" t="inlineStr"/>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>LA 24-20 PHI</t>
+        </is>
+      </c>
+      <c r="N83" t="n">
+        <v>0.909</v>
+      </c>
       <c r="O83" t="inlineStr"/>
       <c r="P83" t="inlineStr"/>
       <c r="Q83" t="inlineStr">
@@ -6025,9 +6205,19 @@
       <c r="K86" t="n">
         <v>58.1</v>
       </c>
-      <c r="L86" t="inlineStr"/>
-      <c r="M86" t="inlineStr"/>
-      <c r="N86" t="inlineStr"/>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>LAC 23-30 SEA</t>
+        </is>
+      </c>
+      <c r="N86" t="n">
+        <v>0</v>
+      </c>
       <c r="O86" t="inlineStr"/>
       <c r="P86" t="inlineStr"/>
       <c r="Q86" t="inlineStr">
@@ -6153,9 +6343,19 @@
       <c r="K88" t="n">
         <v>87.3</v>
       </c>
-      <c r="L88" t="inlineStr"/>
-      <c r="M88" t="inlineStr"/>
-      <c r="N88" t="inlineStr"/>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>LAC 23-30 SEA</t>
+        </is>
+      </c>
+      <c r="N88" t="n">
+        <v>-1</v>
+      </c>
       <c r="O88" t="inlineStr"/>
       <c r="P88" t="inlineStr"/>
       <c r="Q88" t="inlineStr">
@@ -6411,9 +6611,19 @@
       <c r="K92" t="n">
         <v>66.59999999999999</v>
       </c>
-      <c r="L92" t="inlineStr"/>
-      <c r="M92" t="inlineStr"/>
-      <c r="N92" t="inlineStr"/>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>NE 29-26 BUF</t>
+        </is>
+      </c>
+      <c r="N92" t="n">
+        <v>0.909</v>
+      </c>
       <c r="O92" t="inlineStr"/>
       <c r="P92" t="inlineStr"/>
       <c r="Q92" t="inlineStr">
@@ -6539,9 +6749,19 @@
       <c r="K94" t="n">
         <v>77.3</v>
       </c>
-      <c r="L94" t="inlineStr"/>
-      <c r="M94" t="inlineStr"/>
-      <c r="N94" t="inlineStr"/>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>NE 29-26 BUF</t>
+        </is>
+      </c>
+      <c r="N94" t="n">
+        <v>0.909</v>
+      </c>
       <c r="O94" t="inlineStr"/>
       <c r="P94" t="inlineStr"/>
       <c r="Q94" t="inlineStr">
@@ -6732,9 +6952,19 @@
       <c r="K97" t="n">
         <v>70.3</v>
       </c>
-      <c r="L97" t="inlineStr"/>
-      <c r="M97" t="inlineStr"/>
-      <c r="N97" t="inlineStr"/>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>NYJ 12-23 CHI</t>
+        </is>
+      </c>
+      <c r="N97" t="n">
+        <v>0.909</v>
+      </c>
       <c r="O97" t="inlineStr"/>
       <c r="P97" t="inlineStr"/>
       <c r="Q97" t="inlineStr">
@@ -7341,9 +7571,19 @@
       <c r="K106" t="n">
         <v>62.7</v>
       </c>
-      <c r="L106" t="inlineStr"/>
-      <c r="M106" t="inlineStr"/>
-      <c r="N106" t="inlineStr"/>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>TEN 18-24 BAL</t>
+        </is>
+      </c>
+      <c r="N106" t="n">
+        <v>-1</v>
+      </c>
       <c r="O106" t="inlineStr"/>
       <c r="P106" t="inlineStr"/>
       <c r="Q106" t="inlineStr">
@@ -7469,9 +7709,19 @@
       <c r="K108" t="n">
         <v>69.90000000000001</v>
       </c>
-      <c r="L108" t="inlineStr"/>
-      <c r="M108" t="inlineStr"/>
-      <c r="N108" t="inlineStr"/>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>TEN 18-24 BAL</t>
+        </is>
+      </c>
+      <c r="N108" t="n">
+        <v>-1</v>
+      </c>
       <c r="O108" t="inlineStr"/>
       <c r="P108" t="inlineStr"/>
       <c r="Q108" t="inlineStr">
@@ -7675,19 +7925,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E4" t="n">
         <v>2</v>
       </c>
       <c r="G4" t="n">
-        <v>-3.09</v>
+        <v>-3.18</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -7702,22 +7952,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>25</v>
+        <v>47</v>
       </c>
       <c r="C5" t="n">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="D5" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>54.2</v>
+        <v>54.5</v>
       </c>
       <c r="G5" t="n">
-        <v>0.82</v>
+        <v>1.82</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -7732,10 +7982,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -7747,7 +7997,7 @@
         <v>100</v>
       </c>
       <c r="G6" t="n">
-        <v>0.72</v>
+        <v>1.08</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -7987,19 +8237,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D15" t="n">
         <v>3</v>
       </c>
       <c r="E15" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G15" t="n">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -8190,13 +8440,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C27" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D27" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
@@ -8205,7 +8455,7 @@
         <v>50</v>
       </c>
       <c r="G27" t="n">
-        <v>-6.79</v>
+        <v>-7.44</v>
       </c>
       <c r="H27" t="inlineStr"/>
     </row>
@@ -8216,22 +8466,22 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C28" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D28" t="n">
         <v>5</v>
       </c>
       <c r="E28" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F28" t="n">
-        <v>37.5</v>
+        <v>44.4</v>
       </c>
       <c r="G28" t="n">
-        <v>-2.27</v>
+        <v>-1.36</v>
       </c>
       <c r="H28" t="inlineStr"/>
     </row>
@@ -8242,22 +8492,22 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C29" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D29" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>52.9</v>
+        <v>47.6</v>
       </c>
       <c r="G29" t="n">
-        <v>0.18</v>
+        <v>-1.91</v>
       </c>
       <c r="H29" t="inlineStr"/>
     </row>
@@ -8268,22 +8518,22 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="C30" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="D30" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E30" t="n">
         <v>1</v>
       </c>
       <c r="F30" t="n">
-        <v>47.4</v>
+        <v>54.3</v>
       </c>
       <c r="G30" t="n">
-        <v>-1.82</v>
+        <v>1.27</v>
       </c>
       <c r="H30" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
6주차 공식 채점(weekly.py --grade 6) + DAL@GB 발행·보완
- 채점: 시장 7-7 · 발행 6-6 · 모델 6-8 · 관심 ML 2-1(+0.19u) · 시즌 시장 55-37
- picks.csv · predictions.csv · 추적기 xlsx · 6주차 보드(MNF SF 23-17 반영)
- 발행-1018-1635-DALGB(Alijah Clark 제자리 정정) · 발행-1018-1711-보완-DALGB

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/NFL_픽_추적기.xlsx
+++ b/data/NFL_픽_추적기.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q194"/>
+  <dimension ref="A1:Q198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -12147,25 +12147,23 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>ARI@LA</t>
+          <t>BAL@CLE</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>spread</t>
+          <t>ml</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>LA -12.5</t>
-        </is>
-      </c>
-      <c r="E174" t="n">
-        <v>-12.5</v>
-      </c>
+          <t>CLE ML</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr"/>
       <c r="F174" t="inlineStr">
         <is>
-          <t>-110</t>
+          <t>+142</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
@@ -12175,26 +12173,34 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>관찰(큰 괴리 — 페이퍼)</t>
-        </is>
-      </c>
-      <c r="I174" t="n">
-        <v>16.2</v>
-      </c>
-      <c r="J174" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="K174" t="n">
-        <v>61.3</v>
-      </c>
-      <c r="L174" t="inlineStr"/>
-      <c r="M174" t="inlineStr"/>
-      <c r="N174" t="inlineStr"/>
+          <t>각도 관찰 A8(접전 .750+ 팀 → 그 팀 ML)</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr"/>
+      <c r="J174" t="inlineStr"/>
+      <c r="K174" t="inlineStr"/>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M174" t="inlineStr">
+        <is>
+          <t>BAL 10-13 CLE</t>
+        </is>
+      </c>
+      <c r="N174" t="n">
+        <v>1.42</v>
+      </c>
       <c r="O174" t="inlineStr"/>
-      <c r="P174" t="inlineStr"/>
+      <c r="P174" t="inlineStr">
+        <is>
+          <t>CLE 한 포제션 경기 3-1(75%) · 10-18 09:02 PT 판</t>
+        </is>
+      </c>
       <c r="Q174" t="inlineStr">
         <is>
-          <t>2026_06_ARI_LA:spread</t>
+          <t>2026_06_BAL_CLE:ml:A8</t>
         </is>
       </c>
     </row>
@@ -12204,21 +12210,21 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>ARI@LA</t>
+          <t>BAL@CLE</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>total</t>
+          <t>spread</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Over 51.5</t>
+          <t>BAL -3</t>
         </is>
       </c>
       <c r="E175" t="n">
-        <v>51.5</v>
+        <v>-3</v>
       </c>
       <c r="F175" t="inlineStr">
         <is>
@@ -12232,26 +12238,34 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>참고</t>
-        </is>
-      </c>
-      <c r="I175" t="n">
-        <v>54.6</v>
-      </c>
-      <c r="J175" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="K175" t="n">
-        <v>61.5</v>
-      </c>
-      <c r="L175" t="inlineStr"/>
-      <c r="M175" t="inlineStr"/>
-      <c r="N175" t="inlineStr"/>
+          <t>각도 관찰 A3(결장 팀 반대 3점+ 이동 → 결장 팀)</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr"/>
+      <c r="J175" t="inlineStr"/>
+      <c r="K175" t="inlineStr"/>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="M175" t="inlineStr">
+        <is>
+          <t>BAL 10-13 CLE</t>
+        </is>
+      </c>
+      <c r="N175" t="n">
+        <v>-1</v>
+      </c>
       <c r="O175" t="inlineStr"/>
-      <c r="P175" t="inlineStr"/>
+      <c r="P175" t="inlineStr">
+        <is>
+          <t>원정 BAL 결장 확정 · 개장 +6.5 → 지금 +3(홈 기준, +3.5점 반대 이동) · 10-18 09:02 PT 판</t>
+        </is>
+      </c>
       <c r="Q175" t="inlineStr">
         <is>
-          <t>2026_06_ARI_LA:total</t>
+          <t>2026_06_BAL_CLE:spread:A3</t>
         </is>
       </c>
     </row>
@@ -12266,20 +12280,18 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>spread</t>
+          <t>ml</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>BUF -5.5</t>
-        </is>
-      </c>
-      <c r="E176" t="n">
-        <v>5.5</v>
-      </c>
+          <t>BUF ML</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr"/>
       <c r="F176" t="inlineStr">
         <is>
-          <t>-110</t>
+          <t>-238</t>
         </is>
       </c>
       <c r="G176" t="inlineStr">
@@ -12289,26 +12301,34 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>관찰(큰 괴리 — 페이퍼)</t>
-        </is>
-      </c>
-      <c r="I176" t="n">
-        <v>-11.9</v>
-      </c>
-      <c r="J176" t="n">
-        <v>-6.4</v>
-      </c>
-      <c r="K176" t="n">
-        <v>68.8</v>
-      </c>
-      <c r="L176" t="inlineStr"/>
-      <c r="M176" t="inlineStr"/>
-      <c r="N176" t="inlineStr"/>
+          <t>각도 관찰 A8(접전 .750+ 팀 → 그 팀 ML)</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr"/>
+      <c r="J176" t="inlineStr"/>
+      <c r="K176" t="inlineStr"/>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M176" t="inlineStr">
+        <is>
+          <t>BUF 33-30 LV</t>
+        </is>
+      </c>
+      <c r="N176" t="n">
+        <v>0.42</v>
+      </c>
       <c r="O176" t="inlineStr"/>
-      <c r="P176" t="inlineStr"/>
+      <c r="P176" t="inlineStr">
+        <is>
+          <t>BUF 한 포제션 경기 3-1(75%) · 10-18 12:19 PT 판</t>
+        </is>
+      </c>
       <c r="Q176" t="inlineStr">
         <is>
-          <t>2026_06_BUF_LV:spread</t>
+          <t>2026_06_BUF_LV:ml:A8</t>
         </is>
       </c>
     </row>
@@ -12318,25 +12338,23 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>CAR@PHI</t>
+          <t>BUF@LV</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>spread</t>
+          <t>ml</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>PHI +1.5</t>
-        </is>
-      </c>
-      <c r="E177" t="n">
-        <v>1.5</v>
-      </c>
+          <t>BUF ML</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr"/>
       <c r="F177" t="inlineStr">
         <is>
-          <t>-110</t>
+          <t>-238</t>
         </is>
       </c>
       <c r="G177" t="inlineStr">
@@ -12346,26 +12364,34 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>관찰(큰 괴리 — 페이퍼)</t>
-        </is>
-      </c>
-      <c r="I177" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="J177" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="K177" t="n">
-        <v>62.9</v>
-      </c>
-      <c r="L177" t="inlineStr"/>
-      <c r="M177" t="inlineStr"/>
-      <c r="N177" t="inlineStr"/>
+          <t>관심(발행)</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr"/>
+      <c r="J177" t="inlineStr"/>
+      <c r="K177" t="inlineStr"/>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M177" t="inlineStr">
+        <is>
+          <t>BUF 33-30 LV</t>
+        </is>
+      </c>
+      <c r="N177" t="n">
+        <v>0.42</v>
+      </c>
       <c r="O177" t="inlineStr"/>
-      <c r="P177" t="inlineStr"/>
+      <c r="P177" t="inlineStr">
+        <is>
+          <t>발행 판단 소액 관심</t>
+        </is>
+      </c>
       <c r="Q177" t="inlineStr">
         <is>
-          <t>2026_06_CAR_PHI:spread</t>
+          <t>2026_06_BUF_LV:ml:J</t>
         </is>
       </c>
     </row>
@@ -12380,16 +12406,16 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>total</t>
+          <t>spread</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>Over 39.5</t>
+          <t>PHI +3</t>
         </is>
       </c>
       <c r="E178" t="n">
-        <v>39.5</v>
+        <v>3</v>
       </c>
       <c r="F178" t="inlineStr">
         <is>
@@ -12403,26 +12429,34 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>관찰(큰 괴리 — 페이퍼)</t>
-        </is>
-      </c>
-      <c r="I178" t="n">
-        <v>47.2</v>
-      </c>
-      <c r="J178" t="n">
-        <v>7.7</v>
-      </c>
-      <c r="K178" t="n">
-        <v>76.90000000000001</v>
-      </c>
-      <c r="L178" t="inlineStr"/>
-      <c r="M178" t="inlineStr"/>
-      <c r="N178" t="inlineStr"/>
+          <t>각도 관찰 A3(결장 팀 반대 3점+ 이동 → 결장 팀)</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr"/>
+      <c r="J178" t="inlineStr"/>
+      <c r="K178" t="inlineStr"/>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="M178" t="inlineStr">
+        <is>
+          <t>CAR 25-14 PHI</t>
+        </is>
+      </c>
+      <c r="N178" t="n">
+        <v>-1</v>
+      </c>
       <c r="O178" t="inlineStr"/>
-      <c r="P178" t="inlineStr"/>
+      <c r="P178" t="inlineStr">
+        <is>
+          <t>홈 PHI 결장 확정 · 개장 -6.5 → 지금 +3(홈 기준, +9.5점 반대 이동) · 10-18 09:02 PT 판</t>
+        </is>
+      </c>
       <c r="Q178" t="inlineStr">
         <is>
-          <t>2026_06_CAR_PHI:total</t>
+          <t>2026_06_CAR_PHI:spread:A3</t>
         </is>
       </c>
     </row>
@@ -12432,7 +12466,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>CHI@ATL</t>
+          <t>CAR@PHI</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -12442,11 +12476,11 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>ATL +1.5</t>
+          <t>CAR -3</t>
         </is>
       </c>
       <c r="E179" t="n">
-        <v>1.5</v>
+        <v>-3</v>
       </c>
       <c r="F179" t="inlineStr">
         <is>
@@ -12460,26 +12494,34 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>관찰(큰 괴리 — 페이퍼)</t>
-        </is>
-      </c>
-      <c r="I179" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="J179" t="n">
-        <v>6.2</v>
-      </c>
-      <c r="K179" t="n">
-        <v>68.40000000000001</v>
-      </c>
-      <c r="L179" t="inlineStr"/>
-      <c r="M179" t="inlineStr"/>
-      <c r="N179" t="inlineStr"/>
+          <t>새 정보(판 이전·대조)</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr"/>
+      <c r="J179" t="inlineStr"/>
+      <c r="K179" t="inlineStr"/>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>CAR 25-14 PHI</t>
+        </is>
+      </c>
+      <c r="N179" t="n">
+        <v>0.909</v>
+      </c>
       <c r="O179" t="inlineStr"/>
-      <c r="P179" t="inlineStr"/>
+      <c r="P179" t="inlineStr">
+        <is>
+          <t>새 정보: PHI ★주전 OT Lane Johnson(스냅 100%) 개인 사유 결장 확정 · 발표 08:33 PT · 발표 뒤 라인 이동 +0점</t>
+        </is>
+      </c>
       <c r="Q179" t="inlineStr">
         <is>
-          <t>2026_06_CHI_ATL:spread</t>
+          <t>2026_06_CAR_PHI:spread:NC</t>
         </is>
       </c>
     </row>
@@ -12494,16 +12536,16 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>total</t>
+          <t>spread</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>Under 51.5</t>
+          <t>CHI -1.5</t>
         </is>
       </c>
       <c r="E180" t="n">
-        <v>51.5</v>
+        <v>-1.5</v>
       </c>
       <c r="F180" t="inlineStr">
         <is>
@@ -12517,26 +12559,34 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>관찰(큰 괴리 — 페이퍼)</t>
-        </is>
-      </c>
-      <c r="I180" t="n">
-        <v>44.3</v>
-      </c>
-      <c r="J180" t="n">
-        <v>-7.2</v>
-      </c>
-      <c r="K180" t="n">
-        <v>75.5</v>
-      </c>
-      <c r="L180" t="inlineStr"/>
-      <c r="M180" t="inlineStr"/>
-      <c r="N180" t="inlineStr"/>
+          <t>각도 관찰 A6(키 넘버 3·7 넘긴 이동 → 반대쪽 ATS)</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr"/>
+      <c r="J180" t="inlineStr"/>
+      <c r="K180" t="inlineStr"/>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>CHI 31-23 ATL</t>
+        </is>
+      </c>
+      <c r="N180" t="n">
+        <v>0.909</v>
+      </c>
       <c r="O180" t="inlineStr"/>
-      <c r="P180" t="inlineStr"/>
+      <c r="P180" t="inlineStr">
+        <is>
+          <t>개장 +3 → 지금 +1.5(홈 기준) 키 넘버 넘김 · 이동 반대쪽 · 10-18 09:02 PT 판</t>
+        </is>
+      </c>
       <c r="Q180" t="inlineStr">
         <is>
-          <t>2026_06_CHI_ATL:total</t>
+          <t>2026_06_CHI_ATL:spread:A6</t>
         </is>
       </c>
     </row>
@@ -12551,20 +12601,18 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>spread</t>
+          <t>ml</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>GB -1.5</t>
-        </is>
-      </c>
-      <c r="E181" t="n">
-        <v>-1.5</v>
-      </c>
+          <t>GB ML</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr"/>
       <c r="F181" t="inlineStr">
         <is>
-          <t>-110</t>
+          <t>-108</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
@@ -12574,26 +12622,34 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>관찰(큰 괴리 — 페이퍼)</t>
-        </is>
-      </c>
-      <c r="I181" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="J181" t="n">
-        <v>7</v>
-      </c>
-      <c r="K181" t="n">
-        <v>70.59999999999999</v>
-      </c>
-      <c r="L181" t="inlineStr"/>
-      <c r="M181" t="inlineStr"/>
-      <c r="N181" t="inlineStr"/>
+          <t>각도 관찰 A4(작년 플옵팀 언더독 1~8주 → 그 팀 ML)</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr"/>
+      <c r="J181" t="inlineStr"/>
+      <c r="K181" t="inlineStr"/>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M181" t="inlineStr">
+        <is>
+          <t>DAL 13-23 GB</t>
+        </is>
+      </c>
+      <c r="N181" t="n">
+        <v>0.926</v>
+      </c>
       <c r="O181" t="inlineStr"/>
-      <c r="P181" t="inlineStr"/>
+      <c r="P181" t="inlineStr">
+        <is>
+          <t>작년 플옵팀 GB 언더독(무비그 50% · 상대 DAL 비플옵) · 6주차 · 10-18 16:05 PT 판</t>
+        </is>
+      </c>
       <c r="Q181" t="inlineStr">
         <is>
-          <t>2026_06_DAL_GB:spread</t>
+          <t>2026_06_DAL_GB:ml:A4</t>
         </is>
       </c>
     </row>
@@ -12608,16 +12664,16 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>total</t>
+          <t>spread</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>Over 53.5</t>
+          <t>GB +1.5</t>
         </is>
       </c>
       <c r="E182" t="n">
-        <v>53.5</v>
+        <v>1.5</v>
       </c>
       <c r="F182" t="inlineStr">
         <is>
@@ -12631,26 +12687,34 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>관찰(큰 괴리 — 페이퍼)</t>
-        </is>
-      </c>
-      <c r="I182" t="n">
-        <v>64.09999999999999</v>
-      </c>
-      <c r="J182" t="n">
-        <v>10.6</v>
-      </c>
-      <c r="K182" t="n">
-        <v>84.40000000000001</v>
-      </c>
-      <c r="L182" t="inlineStr"/>
-      <c r="M182" t="inlineStr"/>
-      <c r="N182" t="inlineStr"/>
+          <t>각도 관찰 A6(키 넘버 3·7 넘긴 이동 → 반대쪽 ATS)</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr"/>
+      <c r="J182" t="inlineStr"/>
+      <c r="K182" t="inlineStr"/>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>DAL 13-23 GB</t>
+        </is>
+      </c>
+      <c r="N182" t="n">
+        <v>0.909</v>
+      </c>
       <c r="O182" t="inlineStr"/>
-      <c r="P182" t="inlineStr"/>
+      <c r="P182" t="inlineStr">
+        <is>
+          <t>개장 -3 → 지금 +1.5(홈 기준) 키 넘버 넘김 · 이동 반대쪽 · 10-18 16:05 PT 판</t>
+        </is>
+      </c>
       <c r="Q182" t="inlineStr">
         <is>
-          <t>2026_06_DAL_GB:total</t>
+          <t>2026_06_DAL_GB:spread:A6</t>
         </is>
       </c>
     </row>
@@ -12660,7 +12724,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>LAC@KC</t>
+          <t>DAL@GB</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -12670,11 +12734,11 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>LAC +8.5</t>
+          <t>GB +1.5</t>
         </is>
       </c>
       <c r="E183" t="n">
-        <v>8.5</v>
+        <v>1.5</v>
       </c>
       <c r="F183" t="inlineStr">
         <is>
@@ -12694,18 +12758,28 @@
       <c r="I183" t="inlineStr"/>
       <c r="J183" t="inlineStr"/>
       <c r="K183" t="inlineStr"/>
-      <c r="L183" t="inlineStr"/>
-      <c r="M183" t="inlineStr"/>
-      <c r="N183" t="inlineStr"/>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>DAL 13-23 GB</t>
+        </is>
+      </c>
+      <c r="N183" t="n">
+        <v>0.909</v>
+      </c>
       <c r="O183" t="inlineStr"/>
       <c r="P183" t="inlineStr">
         <is>
-          <t>원정 LAC 결장 확정 · 개장 -2.5 → 지금 -8.5(홈 기준, +6점 반대 이동) · 10-14 16:40 PT 판</t>
+          <t>홈 GB 결장 확정 · 개장 -3 → 지금 +1.5(홈 기준, +4.5점 반대 이동) · 10-18 16:05 PT 판</t>
         </is>
       </c>
       <c r="Q183" t="inlineStr">
         <is>
-          <t>2026_06_LAC_KC:spread:A3</t>
+          <t>2026_06_DAL_GB:spread:A3</t>
         </is>
       </c>
     </row>
@@ -12715,7 +12789,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>NO@NYG</t>
+          <t>HOU@JAX</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -12725,11 +12799,11 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>NYG +1.5</t>
+          <t>HOU +2.5</t>
         </is>
       </c>
       <c r="E184" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="F184" t="inlineStr">
         <is>
@@ -12743,26 +12817,34 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>관찰(큰 괴리 — 페이퍼)</t>
-        </is>
-      </c>
-      <c r="I184" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="J184" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="K184" t="n">
-        <v>61.3</v>
-      </c>
-      <c r="L184" t="inlineStr"/>
-      <c r="M184" t="inlineStr"/>
-      <c r="N184" t="inlineStr"/>
+          <t>각도 관찰 A3(결장 팀 반대 3점+ 이동 → 결장 팀)</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr"/>
+      <c r="J184" t="inlineStr"/>
+      <c r="K184" t="inlineStr"/>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>HOU 34-31 JAX</t>
+        </is>
+      </c>
+      <c r="N184" t="n">
+        <v>0.909</v>
+      </c>
       <c r="O184" t="inlineStr"/>
-      <c r="P184" t="inlineStr"/>
+      <c r="P184" t="inlineStr">
+        <is>
+          <t>원정 HOU 결장 확정 · 개장 +1.5 → 지금 -2.5(홈 기준, +4점 반대 이동) · 10-17 19:12 PT 판</t>
+        </is>
+      </c>
       <c r="Q184" t="inlineStr">
         <is>
-          <t>2026_06_NO_NYG:spread</t>
+          <t>2026_06_HOU_JAX:spread:A3</t>
         </is>
       </c>
     </row>
@@ -12772,25 +12854,23 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>NO@NYG</t>
+          <t>LAC@KC</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>spread</t>
+          <t>ml</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>NO -1.5</t>
-        </is>
-      </c>
-      <c r="E185" t="n">
-        <v>-1.5</v>
-      </c>
+          <t>LAC ML</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr"/>
       <c r="F185" t="inlineStr">
         <is>
-          <t>-110</t>
+          <t>+330</t>
         </is>
       </c>
       <c r="G185" t="inlineStr">
@@ -12800,24 +12880,34 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>각도 관찰 A2(드라이브 우위 언더독 반대)</t>
+          <t>각도 관찰 A4(작년 플옵팀 언더독 1~8주 → 그 팀 ML)</t>
         </is>
       </c>
       <c r="I185" t="inlineStr"/>
       <c r="J185" t="inlineStr"/>
       <c r="K185" t="inlineStr"/>
-      <c r="L185" t="inlineStr"/>
-      <c r="M185" t="inlineStr"/>
-      <c r="N185" t="inlineStr"/>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="M185" t="inlineStr">
+        <is>
+          <t>LAC 6-22 KC</t>
+        </is>
+      </c>
+      <c r="N185" t="n">
+        <v>-1</v>
+      </c>
       <c r="O185" t="inlineStr"/>
       <c r="P185" t="inlineStr">
         <is>
-          <t>언더독 NYG 드라이브 득점 차 우위 +0.51 → 반대 NO · 10-14 16:40 PT 판</t>
+          <t>작년 플옵팀 LAC 언더독(무비그 22% · 상대 KC 비플옵) · 6주차 · 10-18 12:19 PT 판</t>
         </is>
       </c>
       <c r="Q185" t="inlineStr">
         <is>
-          <t>2026_06_NO_NYG:spread:A2</t>
+          <t>2026_06_LAC_KC:ml:A4</t>
         </is>
       </c>
     </row>
@@ -12827,25 +12917,23 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>NYJ@NE</t>
+          <t>LAC@KC</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>spread</t>
+          <t>ml</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>NE -7.5</t>
-        </is>
-      </c>
-      <c r="E186" t="n">
-        <v>-7.5</v>
-      </c>
+          <t>KC ML</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr"/>
       <c r="F186" t="inlineStr">
         <is>
-          <t>-110</t>
+          <t>-425</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
@@ -12855,26 +12943,34 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>관찰(큰 괴리 — 페이퍼)</t>
-        </is>
-      </c>
-      <c r="I186" t="n">
-        <v>17.1</v>
-      </c>
-      <c r="J186" t="n">
-        <v>9.6</v>
-      </c>
-      <c r="K186" t="n">
-        <v>76.90000000000001</v>
-      </c>
-      <c r="L186" t="inlineStr"/>
-      <c r="M186" t="inlineStr"/>
-      <c r="N186" t="inlineStr"/>
+          <t>각도 관찰 A5(3rd down 운 회귀 5~9주 → 상대 ML)</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr"/>
+      <c r="J186" t="inlineStr"/>
+      <c r="K186" t="inlineStr"/>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M186" t="inlineStr">
+        <is>
+          <t>LAC 6-22 KC</t>
+        </is>
+      </c>
+      <c r="N186" t="n">
+        <v>0.235</v>
+      </c>
       <c r="O186" t="inlineStr"/>
-      <c r="P186" t="inlineStr"/>
+      <c r="P186" t="inlineStr">
+        <is>
+          <t>LAC 3rd down 21위 vs 공격 EPA 32위(+11) → 상대 KC · 6주차 · 10-18 12:19 PT 판</t>
+        </is>
+      </c>
       <c r="Q186" t="inlineStr">
         <is>
-          <t>2026_06_NYJ_NE:spread</t>
+          <t>2026_06_LAC_KC:ml:A5</t>
         </is>
       </c>
     </row>
@@ -12884,21 +12980,21 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>NYJ@NE</t>
+          <t>LAC@KC</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>total</t>
+          <t>spread</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Over 43.5</t>
+          <t>LAC +7.5</t>
         </is>
       </c>
       <c r="E187" t="n">
-        <v>43.5</v>
+        <v>7.5</v>
       </c>
       <c r="F187" t="inlineStr">
         <is>
@@ -12912,26 +13008,34 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>관찰(큰 괴리 — 페이퍼)</t>
-        </is>
-      </c>
-      <c r="I187" t="n">
-        <v>50.1</v>
-      </c>
-      <c r="J187" t="n">
-        <v>6.6</v>
-      </c>
-      <c r="K187" t="n">
-        <v>73.59999999999999</v>
-      </c>
-      <c r="L187" t="inlineStr"/>
-      <c r="M187" t="inlineStr"/>
-      <c r="N187" t="inlineStr"/>
+          <t>각도 관찰 A3(결장 팀 반대 3점+ 이동 → 결장 팀)</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr"/>
+      <c r="J187" t="inlineStr"/>
+      <c r="K187" t="inlineStr"/>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="M187" t="inlineStr">
+        <is>
+          <t>LAC 6-22 KC</t>
+        </is>
+      </c>
+      <c r="N187" t="n">
+        <v>-1</v>
+      </c>
       <c r="O187" t="inlineStr"/>
-      <c r="P187" t="inlineStr"/>
+      <c r="P187" t="inlineStr">
+        <is>
+          <t>원정 LAC 결장 확정 · 개장 -2.5 → 지금 -7.5(홈 기준, +5점 반대 이동) · 10-18 12:19 PT 판</t>
+        </is>
+      </c>
       <c r="Q187" t="inlineStr">
         <is>
-          <t>2026_06_NYJ_NE:total</t>
+          <t>2026_06_LAC_KC:spread:A3</t>
         </is>
       </c>
     </row>
@@ -12941,7 +13045,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>PIT@TB</t>
+          <t>LAC@KC</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -12951,11 +13055,11 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>TB +2.5</t>
+          <t>LAC +7.5</t>
         </is>
       </c>
       <c r="E188" t="n">
-        <v>2.5</v>
+        <v>7.5</v>
       </c>
       <c r="F188" t="inlineStr">
         <is>
@@ -12969,24 +13073,34 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>각도 관찰 A3(결장 팀 반대 3점+ 이동 → 결장 팀)</t>
+          <t>각도 관찰 A6(키 넘버 3·7 넘긴 이동 → 반대쪽 ATS)</t>
         </is>
       </c>
       <c r="I188" t="inlineStr"/>
       <c r="J188" t="inlineStr"/>
       <c r="K188" t="inlineStr"/>
-      <c r="L188" t="inlineStr"/>
-      <c r="M188" t="inlineStr"/>
-      <c r="N188" t="inlineStr"/>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="M188" t="inlineStr">
+        <is>
+          <t>LAC 6-22 KC</t>
+        </is>
+      </c>
+      <c r="N188" t="n">
+        <v>-1</v>
+      </c>
       <c r="O188" t="inlineStr"/>
       <c r="P188" t="inlineStr">
         <is>
-          <t>홈 TB 결장 확정 · 개장 -1.5 → 지금 +2.5(홈 기준, +4점 반대 이동) · 10-14 16:40 PT 판</t>
+          <t>개장 -2.5 → 지금 -7.5(홈 기준) 키 넘버 넘김 · 이동 반대쪽 · 10-18 12:19 PT 판</t>
         </is>
       </c>
       <c r="Q188" t="inlineStr">
         <is>
-          <t>2026_06_PIT_TB:spread:A3</t>
+          <t>2026_06_LAC_KC:spread:A6</t>
         </is>
       </c>
     </row>
@@ -12996,25 +13110,23 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>SEA@DEN</t>
+          <t>NO@NYG</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>spread</t>
+          <t>ml</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>DEN +2.5</t>
-        </is>
-      </c>
-      <c r="E189" t="n">
-        <v>2.5</v>
-      </c>
+          <t>NYG ML</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr"/>
       <c r="F189" t="inlineStr">
         <is>
-          <t>-110</t>
+          <t>-112</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
@@ -13024,26 +13136,34 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>참고</t>
-        </is>
-      </c>
-      <c r="I189" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="J189" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="K189" t="n">
-        <v>58.3</v>
-      </c>
-      <c r="L189" t="inlineStr"/>
-      <c r="M189" t="inlineStr"/>
-      <c r="N189" t="inlineStr"/>
+          <t>각도 관찰 A5(3rd down 운 회귀 5~9주 → 상대 ML)</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr"/>
+      <c r="J189" t="inlineStr"/>
+      <c r="K189" t="inlineStr"/>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>NO 34-27 NYG</t>
+        </is>
+      </c>
+      <c r="N189" t="n">
+        <v>-1</v>
+      </c>
       <c r="O189" t="inlineStr"/>
-      <c r="P189" t="inlineStr"/>
+      <c r="P189" t="inlineStr">
+        <is>
+          <t>NO 3rd down 7위 vs 공격 EPA 23위(+16) → 상대 NYG · 6주차 · 10-18 09:02 PT 판</t>
+        </is>
+      </c>
       <c r="Q189" t="inlineStr">
         <is>
-          <t>2026_06_SEA_DEN:spread</t>
+          <t>2026_06_NO_NYG:ml:A5</t>
         </is>
       </c>
     </row>
@@ -13053,25 +13173,23 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>SEA@DEN</t>
+          <t>NO@NYG</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>total</t>
+          <t>ml</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Under 40.5</t>
-        </is>
-      </c>
-      <c r="E190" t="n">
-        <v>40.5</v>
-      </c>
+          <t>NYG ML</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr"/>
       <c r="F190" t="inlineStr">
         <is>
-          <t>-110</t>
+          <t>-112</t>
         </is>
       </c>
       <c r="G190" t="inlineStr">
@@ -13081,26 +13199,34 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>참고</t>
-        </is>
-      </c>
-      <c r="I190" t="n">
-        <v>37</v>
-      </c>
-      <c r="J190" t="n">
-        <v>-3.5</v>
-      </c>
-      <c r="K190" t="n">
-        <v>63</v>
-      </c>
-      <c r="L190" t="inlineStr"/>
-      <c r="M190" t="inlineStr"/>
-      <c r="N190" t="inlineStr"/>
+          <t>관심(발행)</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr"/>
+      <c r="J190" t="inlineStr"/>
+      <c r="K190" t="inlineStr"/>
+      <c r="L190" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="M190" t="inlineStr">
+        <is>
+          <t>NO 34-27 NYG</t>
+        </is>
+      </c>
+      <c r="N190" t="n">
+        <v>-1</v>
+      </c>
       <c r="O190" t="inlineStr"/>
-      <c r="P190" t="inlineStr"/>
+      <c r="P190" t="inlineStr">
+        <is>
+          <t>발행 판단 소액 관심</t>
+        </is>
+      </c>
       <c r="Q190" t="inlineStr">
         <is>
-          <t>2026_06_SEA_DEN:total</t>
+          <t>2026_06_NO_NYG:ml:J</t>
         </is>
       </c>
     </row>
@@ -13110,7 +13236,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>TEN@IND</t>
+          <t>NO@NYG</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -13120,11 +13246,11 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>IND -7</t>
+          <t>NYG +1.5</t>
         </is>
       </c>
       <c r="E191" t="n">
-        <v>-7</v>
+        <v>1.5</v>
       </c>
       <c r="F191" t="inlineStr">
         <is>
@@ -13138,26 +13264,34 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>관찰(큰 괴리 — 페이퍼)</t>
-        </is>
-      </c>
-      <c r="I191" t="n">
-        <v>13.5</v>
-      </c>
-      <c r="J191" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="K191" t="n">
-        <v>69.2</v>
-      </c>
-      <c r="L191" t="inlineStr"/>
-      <c r="M191" t="inlineStr"/>
-      <c r="N191" t="inlineStr"/>
+          <t>각도 관찰 A3(결장 팀 반대 3점+ 이동 → 결장 팀)</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr"/>
+      <c r="J191" t="inlineStr"/>
+      <c r="K191" t="inlineStr"/>
+      <c r="L191" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="M191" t="inlineStr">
+        <is>
+          <t>NO 34-27 NYG</t>
+        </is>
+      </c>
+      <c r="N191" t="n">
+        <v>-1</v>
+      </c>
       <c r="O191" t="inlineStr"/>
-      <c r="P191" t="inlineStr"/>
+      <c r="P191" t="inlineStr">
+        <is>
+          <t>홈 NYG 결장 확정 · 개장 -2.5 → 지금 +1.5(홈 기준, +4점 반대 이동) · 10-18 09:02 PT 판</t>
+        </is>
+      </c>
       <c r="Q191" t="inlineStr">
         <is>
-          <t>2026_06_TEN_IND:spread</t>
+          <t>2026_06_NO_NYG:spread:A3</t>
         </is>
       </c>
     </row>
@@ -13167,25 +13301,23 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>TEN@IND</t>
+          <t>PIT@TB</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>spread</t>
+          <t>ml</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>TEN +7</t>
-        </is>
-      </c>
-      <c r="E192" t="n">
-        <v>7</v>
-      </c>
+          <t>PIT ML</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr"/>
       <c r="F192" t="inlineStr">
         <is>
-          <t>-110</t>
+          <t>-130</t>
         </is>
       </c>
       <c r="G192" t="inlineStr">
@@ -13195,24 +13327,34 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>각도 관찰 A3(결장 팀 반대 3점+ 이동 → 결장 팀)</t>
+          <t>각도 관찰 A5(3rd down 운 회귀 5~9주 → 상대 ML)</t>
         </is>
       </c>
       <c r="I192" t="inlineStr"/>
       <c r="J192" t="inlineStr"/>
       <c r="K192" t="inlineStr"/>
-      <c r="L192" t="inlineStr"/>
-      <c r="M192" t="inlineStr"/>
-      <c r="N192" t="inlineStr"/>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M192" t="inlineStr">
+        <is>
+          <t>PIT 26-19 TB</t>
+        </is>
+      </c>
+      <c r="N192" t="n">
+        <v>0.769</v>
+      </c>
       <c r="O192" t="inlineStr"/>
       <c r="P192" t="inlineStr">
         <is>
-          <t>원정 TEN 결장 확정 · 개장 -3.5 → 지금 -7(홈 기준, +3.5점 반대 이동) · 10-14 16:40 PT 판</t>
+          <t>TB 3rd down 16위 vs 공격 EPA 27위(+11) → 상대 PIT · 6주차 · 10-18 09:02 PT 판</t>
         </is>
       </c>
       <c r="Q192" t="inlineStr">
         <is>
-          <t>2026_06_TEN_IND:spread:A3</t>
+          <t>2026_06_PIT_TB:ml:A5</t>
         </is>
       </c>
     </row>
@@ -13222,25 +13364,23 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>WAS@SF</t>
+          <t>PIT@TB</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>spread</t>
+          <t>ml</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>SF -7.5</t>
-        </is>
-      </c>
-      <c r="E193" t="n">
-        <v>-7.5</v>
-      </c>
+          <t>PIT ML</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr"/>
       <c r="F193" t="inlineStr">
         <is>
-          <t>-110</t>
+          <t>-130</t>
         </is>
       </c>
       <c r="G193" t="inlineStr">
@@ -13250,26 +13390,34 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>관찰(큰 괴리 — 페이퍼)</t>
-        </is>
-      </c>
-      <c r="I193" t="n">
-        <v>11.9</v>
-      </c>
-      <c r="J193" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="K193" t="n">
-        <v>63.2</v>
-      </c>
-      <c r="L193" t="inlineStr"/>
-      <c r="M193" t="inlineStr"/>
-      <c r="N193" t="inlineStr"/>
+          <t>관심(발행)</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr"/>
+      <c r="J193" t="inlineStr"/>
+      <c r="K193" t="inlineStr"/>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M193" t="inlineStr">
+        <is>
+          <t>PIT 26-19 TB</t>
+        </is>
+      </c>
+      <c r="N193" t="n">
+        <v>0.769</v>
+      </c>
       <c r="O193" t="inlineStr"/>
-      <c r="P193" t="inlineStr"/>
+      <c r="P193" t="inlineStr">
+        <is>
+          <t>발행 판단 소액 관심</t>
+        </is>
+      </c>
       <c r="Q193" t="inlineStr">
         <is>
-          <t>2026_06_WAS_SF:spread</t>
+          <t>2026_06_PIT_TB:ml:J</t>
         </is>
       </c>
     </row>
@@ -13279,54 +13427,334 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
+          <t>PIT@TB</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>spread</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>TB +1.5</t>
+        </is>
+      </c>
+      <c r="E194" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>-110</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>suggested</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>각도 관찰 A3(결장 팀 반대 3점+ 이동 → 결장 팀)</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr"/>
+      <c r="J194" t="inlineStr"/>
+      <c r="K194" t="inlineStr"/>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="M194" t="inlineStr">
+        <is>
+          <t>PIT 26-19 TB</t>
+        </is>
+      </c>
+      <c r="N194" t="n">
+        <v>-1</v>
+      </c>
+      <c r="O194" t="inlineStr"/>
+      <c r="P194" t="inlineStr">
+        <is>
+          <t>홈 TB 결장 확정 · 개장 -1.5 → 지금 +1.5(홈 기준, +3점 반대 이동) · 10-18 09:02 PT 판</t>
+        </is>
+      </c>
+      <c r="Q194" t="inlineStr">
+        <is>
+          <t>2026_06_PIT_TB:spread:A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>6</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>SEA@DEN</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>spread</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>DEN +2.5</t>
+        </is>
+      </c>
+      <c r="E195" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>-110</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>suggested</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>방향(발행)</t>
+        </is>
+      </c>
+      <c r="I195" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J195" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="K195" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>SEA 14-17 DEN</t>
+        </is>
+      </c>
+      <c r="N195" t="n">
+        <v>0.909</v>
+      </c>
+      <c r="O195" t="inlineStr"/>
+      <c r="P195" t="inlineStr">
+        <is>
+          <t>발행 방향</t>
+        </is>
+      </c>
+      <c r="Q195" t="inlineStr">
+        <is>
+          <t>2026_06_SEA_DEN:spread:D</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>6</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>SEA@DEN</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Under 40.5</t>
+        </is>
+      </c>
+      <c r="E196" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>-110</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>suggested</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>방향(발행)</t>
+        </is>
+      </c>
+      <c r="I196" t="n">
+        <v>37</v>
+      </c>
+      <c r="J196" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="K196" t="n">
+        <v>63</v>
+      </c>
+      <c r="L196" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M196" t="inlineStr">
+        <is>
+          <t>SEA 14-17 DEN</t>
+        </is>
+      </c>
+      <c r="N196" t="n">
+        <v>0.909</v>
+      </c>
+      <c r="O196" t="inlineStr"/>
+      <c r="P196" t="inlineStr">
+        <is>
+          <t>발행 방향</t>
+        </is>
+      </c>
+      <c r="Q196" t="inlineStr">
+        <is>
+          <t>2026_06_SEA_DEN:total:D</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>6</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>TEN@IND</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>spread</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>TEN +6.5</t>
+        </is>
+      </c>
+      <c r="E197" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>-110</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>suggested</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>각도 관찰 A3(결장 팀 반대 3점+ 이동 → 결장 팀)</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr"/>
+      <c r="J197" t="inlineStr"/>
+      <c r="K197" t="inlineStr"/>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M197" t="inlineStr">
+        <is>
+          <t>TEN 26-20 IND</t>
+        </is>
+      </c>
+      <c r="N197" t="n">
+        <v>0.909</v>
+      </c>
+      <c r="O197" t="inlineStr"/>
+      <c r="P197" t="inlineStr">
+        <is>
+          <t>원정 TEN 결장 확정 · 개장 -3.5 → 지금 -6.5(홈 기준, +3점 반대 이동) · 10-18 09:02 PT 판</t>
+        </is>
+      </c>
+      <c r="Q197" t="inlineStr">
+        <is>
+          <t>2026_06_TEN_IND:spread:A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>6</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
           <t>WAS@SF</t>
         </is>
       </c>
-      <c r="C194" t="inlineStr">
-        <is>
-          <t>total</t>
-        </is>
-      </c>
-      <c r="D194" t="inlineStr">
-        <is>
-          <t>Over 50.5</t>
-        </is>
-      </c>
-      <c r="E194" t="n">
-        <v>50.5</v>
-      </c>
-      <c r="F194" t="inlineStr">
-        <is>
-          <t>-110</t>
-        </is>
-      </c>
-      <c r="G194" t="inlineStr">
-        <is>
-          <t>suggested</t>
-        </is>
-      </c>
-      <c r="H194" t="inlineStr">
-        <is>
-          <t>관찰(큰 괴리 — 페이퍼)</t>
-        </is>
-      </c>
-      <c r="I194" t="n">
-        <v>58.3</v>
-      </c>
-      <c r="J194" t="n">
-        <v>7.8</v>
-      </c>
-      <c r="K194" t="n">
-        <v>77.2</v>
-      </c>
-      <c r="L194" t="inlineStr"/>
-      <c r="M194" t="inlineStr"/>
-      <c r="N194" t="inlineStr"/>
-      <c r="O194" t="inlineStr"/>
-      <c r="P194" t="inlineStr"/>
-      <c r="Q194" t="inlineStr">
-        <is>
-          <t>2026_06_WAS_SF:total</t>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>spread</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>WAS +7.5</t>
+        </is>
+      </c>
+      <c r="E198" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>-110</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>suggested</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>각도 관찰 A6(키 넘버 3·7 넘긴 이동 → 반대쪽 ATS)</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr"/>
+      <c r="J198" t="inlineStr"/>
+      <c r="K198" t="inlineStr"/>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>WAS 17-23 SF</t>
+        </is>
+      </c>
+      <c r="N198" t="n">
+        <v>0.909</v>
+      </c>
+      <c r="O198" t="inlineStr"/>
+      <c r="P198" t="inlineStr">
+        <is>
+          <t>개장 -5.5 → 지금 -7.5(홈 기준) 키 넘버 넘김 · 이동 반대쪽 · 10-19 13:23 PT 판</t>
+        </is>
+      </c>
+      <c r="Q198" t="inlineStr">
+        <is>
+          <t>2026_06_WAS_SF:spread:A6</t>
         </is>
       </c>
     </row>
@@ -13427,19 +13855,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
+      <c r="F3" t="n">
+        <v>66.7</v>
+      </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>0.19</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -13454,10 +13885,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C4" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D4" t="n">
         <v>32</v>
@@ -13466,7 +13897,7 @@
         <v>3</v>
       </c>
       <c r="G4" t="n">
-        <v>-11.09</v>
+        <v>-9.27</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -13715,22 +14146,22 @@
         </is>
       </c>
       <c r="B13" t="n">
+        <v>15</v>
+      </c>
+      <c r="C13" t="n">
+        <v>8</v>
+      </c>
+      <c r="D13" t="n">
         <v>7</v>
-      </c>
-      <c r="C13" t="n">
-        <v>5</v>
-      </c>
-      <c r="D13" t="n">
-        <v>2</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>71.40000000000001</v>
+        <v>53.3</v>
       </c>
       <c r="G13" t="n">
-        <v>2.54</v>
+        <v>0.27</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -13796,19 +14227,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C16" t="n">
         <v>11</v>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E16" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G16" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -13999,22 +14430,22 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="C28" t="n">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="D28" t="n">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="E28" t="n">
         <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>50.8</v>
+        <v>53.4</v>
       </c>
       <c r="G28" t="n">
-        <v>-9.94</v>
+        <v>-7.62</v>
       </c>
       <c r="H28" t="inlineStr"/>
     </row>
@@ -14025,10 +14456,10 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C29" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D29" t="n">
         <v>10</v>
@@ -14037,10 +14468,10 @@
         <v>4</v>
       </c>
       <c r="F29" t="n">
-        <v>44.4</v>
+        <v>47.4</v>
       </c>
       <c r="G29" t="n">
-        <v>-2.73</v>
+        <v>-1.82</v>
       </c>
       <c r="H29" t="inlineStr"/>
     </row>
@@ -14051,10 +14482,10 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C30" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D30" t="n">
         <v>16</v>
@@ -14063,10 +14494,10 @@
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>42.9</v>
+        <v>44.8</v>
       </c>
       <c r="G30" t="n">
-        <v>-5.09</v>
+        <v>-4.18</v>
       </c>
       <c r="H30" t="inlineStr"/>
     </row>
@@ -14107,7 +14538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14358,6 +14789,44 @@
         <v>0</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>3</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>